<commit_message>
updates code to add a specific beluga whale exploration
</commit_message>
<xml_diff>
--- a/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
+++ b/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -378,17 +378,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Oncorhynchus keta</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Oncorhynchus kisutch</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>ASV79</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Oncorhynchus keta</t>
+          <t>ASV116</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -397,11 +397,6 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Oncorhynchus spp.</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -425,21 +420,18 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>103</v>
       </c>
       <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
         <v>421</v>
       </c>
-      <c r="G2">
-        <v>71</v>
-      </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>35</v>
-      </c>
-      <c r="J2">
         <v>12</v>
       </c>
     </row>
@@ -461,10 +453,10 @@
         <v>0</v>
       </c>
       <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
         <v>1611</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -475,9 +467,6 @@
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -509,9 +498,6 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
         <v>0</v>
       </c>
     </row>
@@ -522,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -548,17 +534,17 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Oncorhynchus keta</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Oncorhynchus kisutch</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>ASV79</t>
-        </is>
-      </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Oncorhynchus keta</t>
+          <t>ASV116</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -567,11 +553,6 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Oncorhynchus spp.</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -595,22 +576,19 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>0.19216</v>
       </c>
       <c r="F2">
-        <v>0.78108</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>0.13173</v>
+        <v>0.78545</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0.06494</v>
-      </c>
-      <c r="J2">
-        <v>0.02226</v>
+        <v>0.02239</v>
       </c>
     </row>
     <row r="3">
@@ -631,10 +609,10 @@
         <v>0</v>
       </c>
       <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
         <v>0.94431</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -645,9 +623,6 @@
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -679,9 +654,6 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updates all code, figures, etc. to work done all summer (up to 9/28/26; including all work done upon R/V Aquila)
</commit_message>
<xml_diff>
--- a/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
+++ b/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -388,7 +388,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ASV116</t>
+          <t>ASV130</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -397,6 +397,11 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Oncorhynchus spp.</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -420,7 +425,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>103</v>
+        <v>71</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -432,6 +437,9 @@
         <v>0</v>
       </c>
       <c r="I2">
+        <v>35</v>
+      </c>
+      <c r="J2">
         <v>12</v>
       </c>
     </row>
@@ -467,6 +475,9 @@
       <c r="I3">
         <v>0</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -498,6 +509,9 @@
         <v>0</v>
       </c>
       <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
         <v>0</v>
       </c>
     </row>
@@ -508,7 +522,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -544,7 +558,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ASV116</t>
+          <t>ASV130</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -553,6 +567,11 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Oncorhynchus spp.</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -576,19 +595,22 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0.19216</v>
+        <v>0.13173</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0.78545</v>
+        <v>0.78108</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0.02239</v>
+        <v>0.06494</v>
+      </c>
+      <c r="J2">
+        <v>0.02226</v>
       </c>
     </row>
     <row r="3">
@@ -623,6 +645,9 @@
       <c r="I3">
         <v>0</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -654,6 +679,9 @@
         <v>0</v>
       </c>
       <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cleans up update; includes more files
</commit_message>
<xml_diff>
--- a/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
+++ b/Deliverables/12S/regions/cook/ADFG_12s_cook_speciesxsamples.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -388,7 +388,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ASV130</t>
+          <t>ASV116</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -397,11 +397,6 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Oncorhynchus spp.</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -425,7 +420,7 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>71</v>
+        <v>103</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -437,9 +432,6 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>35</v>
-      </c>
-      <c r="J2">
         <v>12</v>
       </c>
     </row>
@@ -475,9 +467,6 @@
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -509,9 +498,6 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
         <v>0</v>
       </c>
     </row>
@@ -522,7 +508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -558,7 +544,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>ASV130</t>
+          <t>ASV116</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -567,11 +553,6 @@
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Oncorhynchus spp.</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Coregonus laurettae</t>
         </is>
@@ -595,22 +576,19 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>0.13173</v>
+        <v>0.19216</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0.78108</v>
+        <v>0.78545</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>0.06494</v>
-      </c>
-      <c r="J2">
-        <v>0.02226</v>
+        <v>0.02239</v>
       </c>
     </row>
     <row r="3">
@@ -645,9 +623,6 @@
       <c r="I3">
         <v>0</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -679,9 +654,6 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
         <v>0</v>
       </c>
     </row>

</xml_diff>